<commit_message>
fix(v6.5.2): Play'n GO 改抓官網 sitemap（含上線日曆）；Kalamba、Casino Inside Romania 改 Firecrawl 輪掃
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sources/igaming-daily-report-sources-v2.xlsx
+++ b/sources/igaming-daily-report-sources-v2.xlsx
@@ -718,12 +718,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Provider 官網</t>
+          <t>Provider 官網；v6.5.2 官網改 Wix、RSS 消失 → 改抓 sitemap（/games/ 的日期＝上線日，/post/ 為新聞）</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>RSS</t>
+          <t>Sitemap</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.playngo.com/blog-feed.xml</t>
+          <t>https://www.playngo.com/sitemap.xml</t>
         </is>
       </c>
     </row>
@@ -1378,22 +1378,22 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Provider 官網</t>
+          <t>Provider 官網；v6.5.2 網站加了機器人驗證（curl 被擋）→ 改 Firecrawl 輪掃</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>WP-API</t>
+          <t>Firecrawl</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>每日</t>
+          <t>輪掃</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://kalambagames.com/wp-json/wp/v2/posts</t>
+          <t>https://kalambagames.com/</t>
         </is>
       </c>
     </row>
@@ -4514,22 +4514,22 @@
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>羅馬尼亞博彩媒體</t>
+          <t>羅馬尼亞博彩媒體；v6.5.2 網站加了機器人驗證（curl 被擋）→ 改 Firecrawl 輪掃</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>WP-API</t>
+          <t>Firecrawl</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>每日</t>
+          <t>輪掃</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>https://casinoinside.ro/wp-json/wp/v2/posts</t>
+          <t>https://casinoinside.ro/</t>
         </is>
       </c>
     </row>

</xml_diff>